<commit_message>
Initial analysis - pull latest changes and understand codebase structure
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TestKit/TestKit/Mapping.xlsx
+++ b/TestKit/TestKit/Mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\School\NET\auto-grading\TestKit\TestKit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C7913F-F082-48BA-A7F0-E8BE65FB8D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2310D547-C715-455E-8404-B087AB1532E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5472" yWindow="2508" windowWidth="17268" windowHeight="9036" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -356,9 +356,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="3" max="3" width="10.19921875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>